<commit_message>
The harness design has been finalized based on a two-connector configuration using 14-pin and 4-pin connectors.
</commit_message>
<xml_diff>
--- a/rover_harness_bom_plan2_4p14p.xlsx
+++ b/rover_harness_bom_plan2_4p14p.xlsx
@@ -24,12 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="264">
-  <si>
-    <t xml:space="preserve">案2：4極＋14極コネクタ（ハーネスは1本）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ハーネス構成（前後間）。端子・ケーブル・材料は両案共通。比較のための資料</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="276">
+  <si>
+    <t xml:space="preserve">案2：4極＋14極コネクタ（ハーネスは1本）【採用】</t>
+  </si>
+  <si>
+    <t xml:space="preserve">採用案。このファイルを正式な購入リストとする。端子・ケーブル・材料は案1と共通</t>
   </si>
   <si>
     <t xml:space="preserve">コネクタ</t>
@@ -665,7 +665,7 @@
     <t xml:space="preserve">③後部ユニット＝メス(5557)、②ハーネス後部側＝オス(5559)、②ハーネス前部側＝メス(5557)、①前部ユニット＝オス(5559)</t>
   </si>
   <si>
-    <t xml:space="preserve">ハーネス部品 購入リスト（Molex Mini-Fit Jr. 版）</t>
+    <t xml:space="preserve">ハーネス部品 購入リスト（Molex Mini-Fit Jr. 4極＋14極 構成・採用版）</t>
   </si>
   <si>
     <t xml:space="preserve">「必要数」「購入数」は式で計算されます。「確認」「購入」列はプルダウンで選択、「実際に購入した品番」は手入力してください。</t>
@@ -2546,7 +2546,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2m</t>
+      <t xml:space="preserve">5m</t>
     </r>
     <r>
       <rPr>
@@ -2563,15 +2563,28 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">34956381</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">。</t>
+      <t xml:space="preserve">34956862</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5mm²×7対、編組シールド＋ドレインワイヤ、絶縁体外径1.5mm、仕上外径9.9mm、許容電流5.4A、150V</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">巻（</t>
     </r>
     <r>
       <rPr>
@@ -2588,17 +2601,14 @@
         <rFont val="Noto Sans CJK SC"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">巻は同ページで選択）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">0.5mm²×7対、編組シールド＋ドレインワイヤ、絶縁体外径1.5mm、仕上外径9.9mm、許容電流5.4A、150V</t>
+      <t xml:space="preserve">）</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">ペア1：RC右＋信号GND、ペア2：RC左＋信号GND、ペア3：5V＋GND、ペア4：SW COM＋NC、ペア5：LED＋＋LED−、ペア6：CURRENT＋VOLTAGE、ペア7：5V＋GND（2本目）。芯線の色をピン配置シートに記録。信号GNDは2本を1端子にダブル圧着</t>
   </si>
   <si>
-    <t xml:space="preserve">必要量1.2m（1台分）は2m巻で満たす。作り直し分も見込むなら5m巻（注文コードは商品ページで確認）</t>
+    <t xml:space="preserve">5m巻×1（1台分の必要量は約1.2m。作り直し・予備を含む）。税別9,498円、出荷6日以内。2m巻（34956381）でも1台分は可</t>
   </si>
   <si>
     <t xml:space="preserve">材料</t>
@@ -2879,6 +2889,122 @@
   </si>
   <si>
     <t xml:space="preserve">AV線が赤黒2色のみのため左右の区別に使用。「前部」「後部」は布テープ（No.16）に記入</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC用 細線（ピグテール）</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">UL1007 AWG24 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">より線（例）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">MDDS30のRC1・RC2の直前でSX(NE)の0.5sq線から継ぐ短い線。信号2本＋GND2本、各5〜10cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SX(NE)の線とはんだで継ぎ、熱収縮チューブ（No.15の1.5／2.5mm）で絶縁。ドレインはこの継ぎ目でGND側の線にはんだ付け（RC1またはRC2の一方のみ）。継ぎ目はMDDS30近くで固定</t>
+  </si>
+  <si>
+    <t xml:space="preserve">手持ちがあれば購入不要。色はSIG／GNDで分けると誤配線防止になる</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dupont 1×3ピン ハウジング＋メス端子</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.54mm</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ピッチ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1×3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ハウジング、メス圧着端子（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AWG22</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">28</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">MDDS30のRC1・RC2（SIG・5V・GNDの3ピン）用。中央の5Vは空き</t>
+  </si>
+  <si>
+    <t xml:space="preserve">組</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IWISS SN-2549で圧着。逆挿し防止のためハウジングとMDDS30にGND側の印、RC1／RC2（R／L）の印を付ける。振動で抜けないようホットボンド等で固定</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ハウジング2個＋端子4個（予備含め多めに）。手持ちのDupontキットがあれば購入不要</t>
   </si>
   <si>
     <t xml:space="preserve">集計</t>
@@ -3470,6 +3596,9 @@
     <t xml:space="preserve">色：オレンジ＝モーター電力、灰＝電源・GND、紫＝アナログ（0〜3.3V）、緑＝RC信号、ピンク＝7S LiPo電圧（電流制限あり）</t>
   </si>
   <si>
+    <t xml:space="preserve">MDDS30側（③）：RC右＝ペア1→RC1のSIG／GND、RC左＝ペア2→RC2のSIG／GND。手前でAWG24に継いでDupont 1×3（中央5Vは空き）。ドレインはRC1かRC2の一方のGNDへ</t>
+  </si>
+  <si>
     <t xml:space="preserve">ハーネス部品 購入リスト：計算条件</t>
   </si>
   <si>
@@ -3486,9 +3615,6 @@
   </si>
   <si>
     <t xml:space="preserve">中継コネクタ位置の数（各サイズとも）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">組</t>
   </si>
   <si>
     <t xml:space="preserve">③-②間、②-①間の2か所。4極・14極それぞれ同数</t>
@@ -4065,7 +4191,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -4127,6 +4253,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4195,6 +4325,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4309,9 +4443,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>241200</xdr:colOff>
+      <xdr:colOff>240840</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>94320</xdr:rowOff>
+      <xdr:rowOff>93960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4325,7 +4459,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="8190720" cy="4475880"/>
+          <a:ext cx="8190360" cy="4475520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4652,7 +4786,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -5417,18 +5551,17 @@
         <v>130</v>
       </c>
       <c r="G21" s="11" t="n">
-        <f aca="false">条件!$B$17</f>
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="H21" s="12" t="n">
-        <f aca="false">ROUNDUP(G21*条件!$B$12,1)</f>
-        <v>2.4</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>102</v>
+        <f aca="false">G21</f>
+        <v>1</v>
+      </c>
+      <c r="I21" s="16" t="s">
+        <v>131</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K21" s="6" t="s">
         <v>44</v>
@@ -5437,7 +5570,7 @@
         <v>45</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5445,19 +5578,19 @@
         <v>14</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G22" s="11" t="n">
         <v>1</v>
@@ -5467,10 +5600,10 @@
         <v>1</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="K22" s="6" t="s">
         <v>44</v>
@@ -5478,8 +5611,8 @@
       <c r="L22" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="M22" s="16" t="s">
-        <v>140</v>
+      <c r="M22" s="17" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5487,19 +5620,19 @@
         <v>15</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>1</v>
@@ -5512,7 +5645,7 @@
         <v>110</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K23" s="6" t="s">
         <v>44</v>
@@ -5521,7 +5654,7 @@
         <v>45</v>
       </c>
       <c r="M23" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5529,19 +5662,19 @@
         <v>16</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G24" s="6" t="n">
         <v>1</v>
@@ -5551,10 +5684,10 @@
         <v>1</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K24" s="6" t="s">
         <v>44</v>
@@ -5563,7 +5696,7 @@
         <v>45</v>
       </c>
       <c r="M24" s="10" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5571,19 +5704,19 @@
         <v>17</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>1</v>
@@ -5593,10 +5726,10 @@
         <v>1</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K25" s="6" t="s">
         <v>44</v>
@@ -5605,7 +5738,7 @@
         <v>45</v>
       </c>
       <c r="M25" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5613,19 +5746,19 @@
         <v>18</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>1</v>
@@ -5635,10 +5768,10 @@
         <v>1</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K26" s="6" t="s">
         <v>44</v>
@@ -5647,66 +5780,150 @@
         <v>45</v>
       </c>
       <c r="M26" s="10" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+        <v>165</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <f aca="false">ROUNDUP(G27*条件!$B$12,1)</f>
+        <v>0.8</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="L27" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="M27" s="10" t="s">
+        <v>170</v>
+      </c>
+    </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="18" t="s">
-        <v>166</v>
-      </c>
-      <c r="C29" s="18" t="str">
-        <f aca="false">COUNTIF(K5:K26,"確認済")&amp;" / "&amp;COUNTA(K5:K26)</f>
-        <v>0 / 22</v>
-      </c>
-    </row>
+      <c r="A28" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <f aca="false">G28</f>
+        <v>2</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="M28" s="10" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="18" t="s">
-        <v>167</v>
-      </c>
-      <c r="C30" s="18" t="str">
-        <f aca="false">COUNTIF(L5:L26,"受領済")&amp;" / "&amp;COUNTA(L5:L26)</f>
-        <v>0 / 22</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+        <v>177</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="C31" s="19" t="str">
+        <f aca="false">COUNTIF(K5:K28,"確認済")&amp;" / "&amp;COUNTA(K5:K28)</f>
+        <v>0 / 24</v>
+      </c>
+    </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="17" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
-        <v>169</v>
-      </c>
-    </row>
+      <c r="A32" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="C32" s="19" t="str">
+        <f aca="false">COUNTIF(L5:L28,"受領済")&amp;" / "&amp;COUNTA(L5:L28)</f>
+        <v>0 / 24</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
-        <v>170</v>
+      <c r="A34" s="18" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>172</v>
+        <v>182</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="3" t="s">
+        <v>184</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K26" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K5:K28" type="list">
       <formula1>"未確認,確認済"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L5:L26" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L5:L28" type="list">
       <formula1>"未購入,発注済,受領済"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5726,7 +5943,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
@@ -5740,553 +5957,558 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
-        <v>173</v>
+      <c r="A1" s="20" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="20" t="s">
-        <v>175</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>176</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>177</v>
-      </c>
-      <c r="E4" s="20" t="s">
+      <c r="B4" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="E4" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="F4" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="G4" s="20" t="s">
+      <c r="F4" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="G4" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="H4" s="20" t="s">
-        <v>179</v>
-      </c>
-      <c r="I4" s="20" t="s">
-        <v>180</v>
+      <c r="H4" s="21" t="s">
+        <v>191</v>
+      </c>
+      <c r="I4" s="21" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>181</v>
-      </c>
-      <c r="B5" s="22" t="n">
+      <c r="A5" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="23" t="s">
-        <v>182</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>183</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>184</v>
-      </c>
-      <c r="F5" s="22" t="s">
-        <v>185</v>
-      </c>
-      <c r="G5" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H5" s="16"/>
-      <c r="I5" s="23" t="s">
-        <v>187</v>
+      <c r="C5" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="D5" s="24" t="s">
+        <v>195</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>196</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="G5" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="H5" s="17"/>
+      <c r="I5" s="24" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>181</v>
-      </c>
-      <c r="B6" s="23" t="n">
+      <c r="A6" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="B6" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="23" t="s">
-        <v>188</v>
-      </c>
-      <c r="D6" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="E6" s="23" t="s">
-        <v>184</v>
-      </c>
-      <c r="F6" s="22" t="s">
-        <v>185</v>
-      </c>
-      <c r="G6" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H6" s="16"/>
-      <c r="I6" s="23" t="s">
-        <v>190</v>
+      <c r="C6" s="24" t="s">
+        <v>200</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>201</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>196</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="G6" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="H6" s="17"/>
+      <c r="I6" s="24" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>181</v>
-      </c>
-      <c r="B7" s="23" t="n">
+      <c r="A7" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="B7" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="23" t="s">
-        <v>182</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>192</v>
-      </c>
-      <c r="F7" s="22" t="s">
-        <v>185</v>
-      </c>
-      <c r="G7" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H7" s="16"/>
-      <c r="I7" s="23" t="s">
+      <c r="C7" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>203</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>204</v>
+      </c>
+      <c r="F7" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="G7" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="H7" s="17"/>
+      <c r="I7" s="24" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="23" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>181</v>
-      </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="C8" s="23" t="s">
-        <v>188</v>
-      </c>
-      <c r="D8" s="23" t="s">
+      <c r="C8" s="24" t="s">
+        <v>200</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>206</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>204</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="H8" s="17"/>
+      <c r="I8" s="24" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="B9" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="26" t="s">
         <v>194</v>
       </c>
-      <c r="E8" s="23" t="s">
-        <v>192</v>
-      </c>
-      <c r="F8" s="22" t="s">
-        <v>185</v>
-      </c>
-      <c r="G8" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H8" s="16"/>
-      <c r="I8" s="23" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="24" t="s">
-        <v>196</v>
-      </c>
-      <c r="B9" s="24" t="n">
+      <c r="D9" s="25" t="s">
+        <v>209</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>210</v>
+      </c>
+      <c r="F9" s="25" t="s">
+        <v>211</v>
+      </c>
+      <c r="G9" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="H9" s="17"/>
+      <c r="I9" s="26" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="B10" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="25" t="s">
-        <v>182</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>197</v>
-      </c>
-      <c r="E9" s="24" t="s">
-        <v>198</v>
-      </c>
-      <c r="F9" s="24" t="s">
-        <v>199</v>
-      </c>
-      <c r="G9" s="24" t="s">
+      <c r="C10" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="H9" s="16"/>
-      <c r="I9" s="25" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24" t="s">
-        <v>196</v>
-      </c>
-      <c r="B10" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="25" t="s">
-        <v>188</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>202</v>
-      </c>
-      <c r="E10" s="24" t="s">
-        <v>198</v>
-      </c>
-      <c r="F10" s="24" t="s">
-        <v>199</v>
-      </c>
-      <c r="G10" s="24" t="s">
+      <c r="D10" s="25" t="s">
+        <v>214</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>210</v>
+      </c>
+      <c r="F10" s="25" t="s">
+        <v>211</v>
+      </c>
+      <c r="G10" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="H10" s="17"/>
+      <c r="I10" s="26" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="B11" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>216</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>210</v>
+      </c>
+      <c r="F11" s="25" t="s">
+        <v>211</v>
+      </c>
+      <c r="G11" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="H11" s="17"/>
+      <c r="I11" s="26" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="B12" s="26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="H10" s="16"/>
-      <c r="I10" s="25" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
-        <v>196</v>
-      </c>
-      <c r="B11" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" s="25" t="s">
-        <v>182</v>
-      </c>
-      <c r="D11" s="24" t="s">
-        <v>204</v>
-      </c>
-      <c r="E11" s="24" t="s">
-        <v>198</v>
-      </c>
-      <c r="F11" s="24" t="s">
-        <v>199</v>
-      </c>
-      <c r="G11" s="24" t="s">
+      <c r="D12" s="25" t="s">
+        <v>218</v>
+      </c>
+      <c r="E12" s="25" t="s">
+        <v>210</v>
+      </c>
+      <c r="F12" s="25" t="s">
+        <v>211</v>
+      </c>
+      <c r="G12" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="H12" s="17"/>
+      <c r="I12" s="26" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="27" t="s">
+        <v>208</v>
+      </c>
+      <c r="B13" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>194</v>
+      </c>
+      <c r="D13" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E13" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="F13" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="G13" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="H13" s="17"/>
+      <c r="I13" s="28" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="27" t="s">
+        <v>208</v>
+      </c>
+      <c r="B14" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="28" t="s">
         <v>200</v>
       </c>
-      <c r="H11" s="16"/>
-      <c r="I11" s="25" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
-        <v>196</v>
-      </c>
-      <c r="B12" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>188</v>
-      </c>
-      <c r="D12" s="24" t="s">
-        <v>206</v>
-      </c>
-      <c r="E12" s="24" t="s">
-        <v>198</v>
-      </c>
-      <c r="F12" s="24" t="s">
-        <v>199</v>
-      </c>
-      <c r="G12" s="24" t="s">
+      <c r="D14" s="27" t="s">
+        <v>222</v>
+      </c>
+      <c r="E14" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="F14" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="G14" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="H14" s="17"/>
+      <c r="I14" s="28" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="29" t="s">
+        <v>208</v>
+      </c>
+      <c r="B15" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="30" t="s">
+        <v>194</v>
+      </c>
+      <c r="D15" s="29" t="s">
+        <v>224</v>
+      </c>
+      <c r="E15" s="29" t="s">
+        <v>210</v>
+      </c>
+      <c r="F15" s="29" t="s">
+        <v>211</v>
+      </c>
+      <c r="G15" s="29" t="s">
+        <v>212</v>
+      </c>
+      <c r="H15" s="17"/>
+      <c r="I15" s="30" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="29" t="s">
+        <v>208</v>
+      </c>
+      <c r="B16" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="30" t="s">
         <v>200</v>
       </c>
-      <c r="H12" s="16"/>
-      <c r="I12" s="25" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="26" t="s">
-        <v>196</v>
-      </c>
-      <c r="B13" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="C13" s="27" t="s">
-        <v>182</v>
-      </c>
-      <c r="D13" s="26" t="s">
+      <c r="D16" s="29" t="s">
+        <v>226</v>
+      </c>
+      <c r="E16" s="29" t="s">
+        <v>210</v>
+      </c>
+      <c r="F16" s="29" t="s">
+        <v>211</v>
+      </c>
+      <c r="G16" s="29" t="s">
+        <v>212</v>
+      </c>
+      <c r="H16" s="17"/>
+      <c r="I16" s="30" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="25" t="s">
         <v>208</v>
       </c>
-      <c r="E13" s="26" t="s">
-        <v>198</v>
-      </c>
-      <c r="F13" s="26" t="s">
-        <v>199</v>
-      </c>
-      <c r="G13" s="26" t="s">
+      <c r="B17" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="D17" s="26" t="s">
+        <v>228</v>
+      </c>
+      <c r="E17" s="25" t="s">
+        <v>210</v>
+      </c>
+      <c r="F17" s="25" t="s">
+        <v>211</v>
+      </c>
+      <c r="G17" s="25" t="s">
+        <v>229</v>
+      </c>
+      <c r="H17" s="17"/>
+      <c r="I17" s="26" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="B18" s="26" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="H13" s="16"/>
-      <c r="I13" s="27" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="26" t="s">
-        <v>196</v>
-      </c>
-      <c r="B14" s="27" t="n">
-        <v>3</v>
-      </c>
-      <c r="C14" s="27" t="s">
-        <v>188</v>
-      </c>
-      <c r="D14" s="26" t="s">
+      <c r="D18" s="26" t="s">
+        <v>231</v>
+      </c>
+      <c r="E18" s="25" t="s">
         <v>210</v>
       </c>
-      <c r="E14" s="26" t="s">
-        <v>198</v>
-      </c>
-      <c r="F14" s="26" t="s">
-        <v>199</v>
-      </c>
-      <c r="G14" s="26" t="s">
+      <c r="F18" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="G18" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="H18" s="17"/>
+      <c r="I18" s="26" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="31" t="s">
+        <v>208</v>
+      </c>
+      <c r="B19" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="D19" s="31" t="s">
+        <v>233</v>
+      </c>
+      <c r="E19" s="31" t="s">
+        <v>210</v>
+      </c>
+      <c r="F19" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="G19" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="H19" s="17"/>
+      <c r="I19" s="32" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="31" t="s">
+        <v>208</v>
+      </c>
+      <c r="B20" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" s="32" t="s">
         <v>200</v>
       </c>
-      <c r="H14" s="16"/>
-      <c r="I14" s="27" t="s">
+      <c r="D20" s="31" t="s">
+        <v>235</v>
+      </c>
+      <c r="E20" s="31" t="s">
+        <v>210</v>
+      </c>
+      <c r="F20" s="31" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="28" t="s">
-        <v>196</v>
-      </c>
-      <c r="B15" s="28" t="n">
-        <v>4</v>
-      </c>
-      <c r="C15" s="29" t="s">
-        <v>182</v>
-      </c>
-      <c r="D15" s="28" t="s">
+      <c r="G20" s="31" t="s">
         <v>212</v>
       </c>
-      <c r="E15" s="28" t="s">
-        <v>198</v>
-      </c>
-      <c r="F15" s="28" t="s">
-        <v>199</v>
-      </c>
-      <c r="G15" s="28" t="s">
+      <c r="H20" s="17"/>
+      <c r="I20" s="32" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="31" t="s">
+        <v>208</v>
+      </c>
+      <c r="B21" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C21" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="D21" s="31" t="s">
+        <v>237</v>
+      </c>
+      <c r="E21" s="31" t="s">
+        <v>210</v>
+      </c>
+      <c r="F21" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="G21" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="H21" s="17"/>
+      <c r="I21" s="32" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="31" t="s">
+        <v>208</v>
+      </c>
+      <c r="B22" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" s="32" t="s">
         <v>200</v>
       </c>
-      <c r="H15" s="16"/>
-      <c r="I15" s="29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
-        <v>196</v>
-      </c>
-      <c r="B16" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="C16" s="29" t="s">
-        <v>188</v>
-      </c>
-      <c r="D16" s="28" t="s">
-        <v>214</v>
-      </c>
-      <c r="E16" s="28" t="s">
-        <v>198</v>
-      </c>
-      <c r="F16" s="28" t="s">
-        <v>199</v>
-      </c>
-      <c r="G16" s="28" t="s">
-        <v>200</v>
-      </c>
-      <c r="H16" s="16"/>
-      <c r="I16" s="29" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="24" t="s">
-        <v>196</v>
-      </c>
-      <c r="B17" s="25" t="n">
-        <v>5</v>
-      </c>
-      <c r="C17" s="25" t="s">
-        <v>182</v>
-      </c>
-      <c r="D17" s="25" t="s">
-        <v>216</v>
-      </c>
-      <c r="E17" s="24" t="s">
-        <v>198</v>
-      </c>
-      <c r="F17" s="24" t="s">
-        <v>199</v>
-      </c>
-      <c r="G17" s="24" t="s">
-        <v>217</v>
-      </c>
-      <c r="H17" s="16"/>
-      <c r="I17" s="25" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="24" t="s">
-        <v>196</v>
-      </c>
-      <c r="B18" s="25" t="n">
-        <v>5</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>188</v>
-      </c>
-      <c r="D18" s="25" t="s">
-        <v>219</v>
-      </c>
-      <c r="E18" s="24" t="s">
-        <v>198</v>
-      </c>
-      <c r="F18" s="24" t="s">
-        <v>122</v>
-      </c>
-      <c r="G18" s="24" t="s">
-        <v>200</v>
-      </c>
-      <c r="H18" s="16"/>
-      <c r="I18" s="25" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="30" t="s">
-        <v>196</v>
-      </c>
-      <c r="B19" s="30" t="n">
-        <v>6</v>
-      </c>
-      <c r="C19" s="31" t="s">
-        <v>182</v>
-      </c>
-      <c r="D19" s="30" t="s">
-        <v>221</v>
-      </c>
-      <c r="E19" s="30" t="s">
-        <v>198</v>
-      </c>
-      <c r="F19" s="30" t="s">
-        <v>199</v>
-      </c>
-      <c r="G19" s="30" t="s">
-        <v>200</v>
-      </c>
-      <c r="H19" s="16"/>
-      <c r="I19" s="31" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="30" t="s">
-        <v>196</v>
-      </c>
-      <c r="B20" s="31" t="n">
-        <v>6</v>
-      </c>
-      <c r="C20" s="31" t="s">
-        <v>188</v>
-      </c>
-      <c r="D20" s="30" t="s">
-        <v>223</v>
-      </c>
-      <c r="E20" s="30" t="s">
-        <v>198</v>
-      </c>
-      <c r="F20" s="30" t="s">
-        <v>199</v>
-      </c>
-      <c r="G20" s="30" t="s">
-        <v>200</v>
-      </c>
-      <c r="H20" s="16"/>
-      <c r="I20" s="31" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="30" t="s">
-        <v>196</v>
-      </c>
-      <c r="B21" s="31" t="n">
-        <v>7</v>
-      </c>
-      <c r="C21" s="31" t="s">
-        <v>182</v>
-      </c>
-      <c r="D21" s="30" t="s">
-        <v>225</v>
-      </c>
-      <c r="E21" s="30" t="s">
-        <v>198</v>
-      </c>
-      <c r="F21" s="30" t="s">
-        <v>199</v>
-      </c>
-      <c r="G21" s="30" t="s">
-        <v>200</v>
-      </c>
-      <c r="H21" s="16"/>
-      <c r="I21" s="31" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="30" t="s">
-        <v>196</v>
-      </c>
-      <c r="B22" s="31" t="n">
-        <v>7</v>
-      </c>
-      <c r="C22" s="31" t="s">
-        <v>188</v>
-      </c>
-      <c r="D22" s="30" t="s">
-        <v>227</v>
-      </c>
-      <c r="E22" s="30" t="s">
-        <v>198</v>
-      </c>
-      <c r="F22" s="30" t="s">
-        <v>199</v>
-      </c>
-      <c r="G22" s="30" t="s">
-        <v>200</v>
-      </c>
-      <c r="H22" s="16"/>
-      <c r="I22" s="31" t="s">
-        <v>228</v>
+      <c r="D22" s="31" t="s">
+        <v>239</v>
+      </c>
+      <c r="E22" s="31" t="s">
+        <v>210</v>
+      </c>
+      <c r="F22" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="G22" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="H22" s="17"/>
+      <c r="I22" s="32" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="32" t="s">
-        <v>230</v>
+      <c r="A25" s="33" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="32" t="s">
-        <v>232</v>
+      <c r="A27" s="33" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>233</v>
+        <v>245</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="34" t="s">
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -6316,194 +6538,194 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
-        <v>236</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>237</v>
-      </c>
-      <c r="C4" s="20" t="s">
+      <c r="A4" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>250</v>
+      </c>
+      <c r="C4" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="20" t="s">
-        <v>238</v>
+      <c r="D4" s="21" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="33" t="s">
-        <v>239</v>
-      </c>
-      <c r="B5" s="34" t="n">
+      <c r="A5" s="35" t="s">
+        <v>252</v>
+      </c>
+      <c r="B5" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="33" t="s">
-        <v>240</v>
-      </c>
-      <c r="D5" s="35" t="s">
-        <v>241</v>
+      <c r="C5" s="35" t="s">
+        <v>174</v>
+      </c>
+      <c r="D5" s="37" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="36" t="s">
-        <v>242</v>
-      </c>
-      <c r="B6" s="34" t="n">
+      <c r="A6" s="38" t="s">
+        <v>254</v>
+      </c>
+      <c r="B6" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="33" t="s">
+      <c r="C6" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="D6" s="35" t="s">
-        <v>243</v>
+      <c r="D6" s="37" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="36" t="s">
-        <v>244</v>
-      </c>
-      <c r="B7" s="34" t="n">
+      <c r="A7" s="38" t="s">
+        <v>256</v>
+      </c>
+      <c r="B7" s="36" t="n">
         <v>14</v>
       </c>
-      <c r="C7" s="33" t="s">
+      <c r="C7" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="D7" s="37" t="s">
-        <v>245</v>
+      <c r="D7" s="39" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="33" t="s">
-        <v>246</v>
-      </c>
-      <c r="B8" s="34" t="n">
+      <c r="A8" s="35" t="s">
+        <v>258</v>
+      </c>
+      <c r="B8" s="36" t="n">
         <v>2.5</v>
       </c>
-      <c r="C8" s="33" t="s">
-        <v>247</v>
-      </c>
-      <c r="D8" s="35" t="s">
-        <v>248</v>
+      <c r="C8" s="35" t="s">
+        <v>259</v>
+      </c>
+      <c r="D8" s="37" t="s">
+        <v>260</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="B9" s="34" t="n">
+      <c r="A9" s="35" t="s">
+        <v>261</v>
+      </c>
+      <c r="B9" s="36" t="n">
         <v>0.6</v>
       </c>
-      <c r="C9" s="36" t="s">
+      <c r="C9" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="D9" s="35" t="s">
-        <v>250</v>
+      <c r="D9" s="37" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="33" t="s">
-        <v>251</v>
-      </c>
-      <c r="B10" s="34" t="n">
+      <c r="A10" s="35" t="s">
+        <v>263</v>
+      </c>
+      <c r="B10" s="36" t="n">
         <v>0.3</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="D10" s="35" t="s">
-        <v>252</v>
+      <c r="D10" s="37" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="33" t="s">
-        <v>253</v>
-      </c>
-      <c r="B11" s="34" t="n">
+      <c r="A11" s="35" t="s">
+        <v>265</v>
+      </c>
+      <c r="B11" s="36" t="n">
         <v>0.3</v>
       </c>
-      <c r="C11" s="36" t="s">
+      <c r="C11" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="D11" s="35" t="s">
-        <v>252</v>
+      <c r="D11" s="37" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="33" t="s">
-        <v>254</v>
-      </c>
-      <c r="B12" s="34" t="n">
+      <c r="A12" s="35" t="s">
+        <v>266</v>
+      </c>
+      <c r="B12" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="33" t="s">
-        <v>247</v>
-      </c>
-      <c r="D12" s="35" t="s">
-        <v>255</v>
+      <c r="C12" s="35" t="s">
+        <v>259</v>
+      </c>
+      <c r="D12" s="37" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="33" t="s">
-        <v>256</v>
-      </c>
-      <c r="B13" s="34" t="n">
+      <c r="A13" s="35" t="s">
+        <v>268</v>
+      </c>
+      <c r="B13" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="D13" s="35" t="s">
-        <v>257</v>
+      <c r="D13" s="37" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="33" t="s">
-        <v>258</v>
-      </c>
-      <c r="B14" s="34" t="n">
+      <c r="A14" s="35" t="s">
+        <v>270</v>
+      </c>
+      <c r="B14" s="36" t="n">
         <v>1.2</v>
       </c>
-      <c r="C14" s="33" t="s">
-        <v>247</v>
-      </c>
-      <c r="D14" s="35" t="s">
+      <c r="C14" s="35" t="s">
         <v>259</v>
       </c>
+      <c r="D14" s="37" t="s">
+        <v>271</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="33" t="s">
-        <v>260</v>
-      </c>
-      <c r="B15" s="34" t="n">
+      <c r="A15" s="35" t="s">
+        <v>272</v>
+      </c>
+      <c r="B15" s="36" t="n">
         <v>6</v>
       </c>
-      <c r="C15" s="33" t="s">
-        <v>261</v>
-      </c>
-      <c r="D15" s="35" t="s">
-        <v>262</v>
+      <c r="C15" s="35" t="s">
+        <v>273</v>
+      </c>
+      <c r="D15" s="37" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38" t="s">
-        <v>263</v>
-      </c>
-      <c r="B17" s="33" t="n">
+      <c r="A17" s="40" t="s">
+        <v>275</v>
+      </c>
+      <c r="B17" s="35" t="n">
         <f aca="false">B9+B10+B11</f>
         <v>1.2</v>
       </c>
-      <c r="C17" s="39" t="s">
+      <c r="C17" s="41" t="s">
         <v>102</v>
       </c>
-      <c r="D17" s="39"/>
+      <c r="D17" s="41"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>